<commit_message>
last minute style changes and fix download button
</commit_message>
<xml_diff>
--- a/data/Fielddata_2024_2025.xlsx
+++ b/data/Fielddata_2024_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emmersonEmmerson/Documents/Master's/Work feb 2025/NL_watersheds/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A871C16-49DB-2C4C-AB5A-5C3387E8C330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E99DAA2-BE44-E44B-B21B-71FCBF19C751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Invertebrate and periphyton" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId5"/>
+    <pivotCache cacheId="5" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -997,50 +997,59 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1048,6 +1057,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1256,17 +1266,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1274,10 +1275,19 @@
     <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1296,7 +1306,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Microsoft Office User" refreshedDate="46086.54079363426" refreshedVersion="8" recordCount="283" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Microsoft Office User" refreshedDate="46094.624591898151" refreshedVersion="8" recordCount="283" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G996" sheet="Temperature"/>
   </cacheSource>
@@ -3905,7 +3915,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="Temperature" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="Temperature" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
   <location ref="I6:L28" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField name="Location" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
@@ -4264,10 +4274,10 @@
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="38" t="s">
+      <c r="F1" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="G1" s="38" t="s">
+      <c r="G1" s="29" t="s">
         <v>307</v>
       </c>
       <c r="H1" s="2" t="s">
@@ -4276,7 +4286,7 @@
       <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="42" t="s">
+      <c r="J1" s="33" t="s">
         <v>6</v>
       </c>
       <c r="K1" s="1"/>
@@ -4335,7 +4345,7 @@
         <v>-56.01231</v>
       </c>
       <c r="G3" s="6" t="str">
-        <f t="shared" ref="G3:G59" si="1">MID(D3,2,8)</f>
+        <f t="shared" ref="G3:G14" si="1">MID(D3,2,8)</f>
         <v>48.89357</v>
       </c>
       <c r="H3" s="7">
@@ -9115,10 +9125,10 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="38" t="s">
+      <c r="E1" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="F1" s="38" t="s">
+      <c r="F1" s="29" t="s">
         <v>307</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -9151,14 +9161,14 @@
       <c r="P1" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="Q1" s="38" t="s">
+      <c r="Q1" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="R1" s="39" t="s">
+      <c r="R1" s="30" t="s">
         <v>309</v>
       </c>
-      <c r="S1" s="40"/>
-      <c r="T1" s="38"/>
+      <c r="S1" s="31"/>
+      <c r="T1" s="29"/>
     </row>
     <row r="2" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
@@ -9219,7 +9229,7 @@
         <f>SUM(L2:P2)</f>
         <v>113</v>
       </c>
-      <c r="S2" s="41"/>
+      <c r="S2" s="32"/>
     </row>
     <row r="3" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
@@ -9280,7 +9290,7 @@
         <f t="shared" ref="R3:R14" si="3">SUM(L3:P3)</f>
         <v>0</v>
       </c>
-      <c r="S3" s="41"/>
+      <c r="S3" s="32"/>
     </row>
     <row r="4" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
@@ -9341,7 +9351,7 @@
         <f t="shared" si="3"/>
         <v>70</v>
       </c>
-      <c r="S4" s="41"/>
+      <c r="S4" s="32"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
@@ -9402,7 +9412,7 @@
         <f t="shared" si="3"/>
         <v>49</v>
       </c>
-      <c r="S5" s="41"/>
+      <c r="S5" s="32"/>
     </row>
     <row r="6" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
@@ -9463,7 +9473,7 @@
         <f t="shared" si="3"/>
         <v>38</v>
       </c>
-      <c r="S6" s="41"/>
+      <c r="S6" s="32"/>
     </row>
     <row r="7" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
@@ -9524,7 +9534,7 @@
         <f t="shared" si="3"/>
         <v>321</v>
       </c>
-      <c r="S7" s="41"/>
+      <c r="S7" s="32"/>
     </row>
     <row r="8" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
@@ -9585,7 +9595,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S8" s="41"/>
+      <c r="S8" s="32"/>
     </row>
     <row r="9" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
@@ -9646,7 +9656,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S9" s="41"/>
+      <c r="S9" s="32"/>
     </row>
     <row r="10" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
@@ -9707,7 +9717,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S10" s="41"/>
+      <c r="S10" s="32"/>
     </row>
     <row r="11" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
@@ -9768,7 +9778,7 @@
         <f t="shared" si="3"/>
         <v>62</v>
       </c>
-      <c r="S11" s="41"/>
+      <c r="S11" s="32"/>
     </row>
     <row r="12" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
@@ -9829,7 +9839,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S12" s="41"/>
+      <c r="S12" s="32"/>
     </row>
     <row r="13" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
@@ -9890,7 +9900,7 @@
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="S13" s="41"/>
+      <c r="S13" s="32"/>
     </row>
     <row r="14" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
@@ -9951,7 +9961,7 @@
         <f t="shared" si="3"/>
         <v>129</v>
       </c>
-      <c r="S14" s="41"/>
+      <c r="S14" s="32"/>
     </row>
     <row r="15" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="R15" s="13"/>
@@ -10297,13 +10307,13 @@
       <c r="I8" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="J8" s="27">
+      <c r="J8" s="34">
         <v>5.7279230769230773</v>
       </c>
-      <c r="K8" s="28">
+      <c r="K8" s="35">
         <v>15.656307692307694</v>
       </c>
-      <c r="L8" s="29">
+      <c r="L8" s="36">
         <v>9.7515887061538482</v>
       </c>
     </row>
@@ -10329,16 +10339,16 @@
       <c r="G9" s="18">
         <v>16.39</v>
       </c>
-      <c r="I9" s="30" t="s">
+      <c r="I9" s="27" t="s">
         <v>208</v>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="37">
         <v>5.2112740389230785</v>
       </c>
-      <c r="K9" s="32">
+      <c r="K9" s="38">
         <v>13.048845402846155</v>
       </c>
-      <c r="L9" s="33">
+      <c r="L9" s="39">
         <v>8.445542115692307</v>
       </c>
     </row>
@@ -10364,16 +10374,16 @@
       <c r="G10" s="18">
         <v>13.34</v>
       </c>
-      <c r="I10" s="30" t="s">
+      <c r="I10" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="J10" s="31">
+      <c r="J10" s="37">
         <v>8.4382352941176482</v>
       </c>
-      <c r="K10" s="32">
+      <c r="K10" s="38">
         <v>16.831176470588236</v>
       </c>
-      <c r="L10" s="33">
+      <c r="L10" s="39">
         <v>11.95817269882353</v>
       </c>
     </row>
@@ -10399,16 +10409,16 @@
       <c r="G11" s="18">
         <v>13.6</v>
       </c>
-      <c r="I11" s="30" t="s">
+      <c r="I11" s="27" t="s">
         <v>210</v>
       </c>
-      <c r="J11" s="31">
+      <c r="J11" s="37">
         <v>5.9446666666666657</v>
       </c>
-      <c r="K11" s="32">
+      <c r="K11" s="38">
         <v>17.786000000000001</v>
       </c>
-      <c r="L11" s="33">
+      <c r="L11" s="39">
         <v>11.007528450466667</v>
       </c>
     </row>
@@ -10434,16 +10444,16 @@
       <c r="G12" s="18">
         <v>14.93</v>
       </c>
-      <c r="I12" s="30" t="s">
+      <c r="I12" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="J12" s="31">
+      <c r="J12" s="37">
         <v>6.2737333333333334</v>
       </c>
-      <c r="K12" s="32">
+      <c r="K12" s="38">
         <v>17.075866666666666</v>
       </c>
-      <c r="L12" s="33">
+      <c r="L12" s="39">
         <v>10.991642688466666</v>
       </c>
     </row>
@@ -10469,16 +10479,16 @@
       <c r="G13" s="18">
         <v>10.85</v>
       </c>
-      <c r="I13" s="30" t="s">
+      <c r="I13" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="J13" s="31">
+      <c r="J13" s="37">
         <v>8.113999999999999</v>
       </c>
-      <c r="K13" s="32">
+      <c r="K13" s="38">
         <v>15.86066666666667</v>
       </c>
-      <c r="L13" s="33">
+      <c r="L13" s="39">
         <v>11.467337102933335</v>
       </c>
     </row>
@@ -10504,16 +10514,16 @@
       <c r="G14" s="18">
         <v>3.9</v>
       </c>
-      <c r="I14" s="30" t="s">
+      <c r="I14" s="27" t="s">
         <v>200</v>
       </c>
-      <c r="J14" s="31">
+      <c r="J14" s="37">
         <v>6.8653333333333331</v>
       </c>
-      <c r="K14" s="32">
+      <c r="K14" s="38">
         <v>16.913333333333334</v>
       </c>
-      <c r="L14" s="33">
+      <c r="L14" s="39">
         <v>11.339476139933332</v>
       </c>
     </row>
@@ -10539,16 +10549,16 @@
       <c r="G15" s="18">
         <v>1.24</v>
       </c>
-      <c r="I15" s="30" t="s">
+      <c r="I15" s="27" t="s">
         <v>213</v>
       </c>
-      <c r="J15" s="31">
+      <c r="J15" s="37">
         <v>5.9013333333333327</v>
       </c>
-      <c r="K15" s="32">
+      <c r="K15" s="38">
         <v>16.605333333333331</v>
       </c>
-      <c r="L15" s="33">
+      <c r="L15" s="39">
         <v>10.33067759926667</v>
       </c>
     </row>
@@ -10574,16 +10584,16 @@
       <c r="G16" s="18">
         <v>0.21</v>
       </c>
-      <c r="I16" s="30" t="s">
+      <c r="I16" s="27" t="s">
         <v>214</v>
       </c>
-      <c r="J16" s="31">
+      <c r="J16" s="37">
         <v>7.4776470588235293</v>
       </c>
-      <c r="K16" s="32">
+      <c r="K16" s="38">
         <v>16.022941176470592</v>
       </c>
-      <c r="L16" s="33">
+      <c r="L16" s="39">
         <v>10.928438752235294</v>
       </c>
     </row>
@@ -10609,16 +10619,16 @@
       <c r="G17" s="18">
         <v>0.34</v>
       </c>
-      <c r="I17" s="30" t="s">
+      <c r="I17" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="J17" s="31">
+      <c r="J17" s="37">
         <v>5.9205384615384613</v>
       </c>
-      <c r="K17" s="32">
+      <c r="K17" s="38">
         <v>15.801769230769231</v>
       </c>
-      <c r="L17" s="33">
+      <c r="L17" s="39">
         <v>9.7896560026153843</v>
       </c>
     </row>
@@ -10644,16 +10654,16 @@
       <c r="G18" s="18">
         <v>0.47</v>
       </c>
-      <c r="I18" s="30" t="s">
+      <c r="I18" s="27" t="s">
         <v>217</v>
       </c>
-      <c r="J18" s="31">
+      <c r="J18" s="37">
         <v>6.7039999999999997</v>
       </c>
-      <c r="K18" s="32">
+      <c r="K18" s="38">
         <v>15.617999999999999</v>
       </c>
-      <c r="L18" s="33">
+      <c r="L18" s="39">
         <v>10.717379217600001</v>
       </c>
     </row>
@@ -10679,16 +10689,16 @@
       <c r="G19" s="18">
         <v>0.9</v>
       </c>
-      <c r="I19" s="30" t="s">
+      <c r="I19" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="J19" s="31">
+      <c r="J19" s="37">
         <v>7.3989739582</v>
       </c>
-      <c r="K19" s="32">
+      <c r="K19" s="38">
         <v>16.082013021200002</v>
       </c>
-      <c r="L19" s="33">
+      <c r="L19" s="39">
         <v>11.113304186533334</v>
       </c>
     </row>
@@ -10714,16 +10724,16 @@
       <c r="G20" s="18">
         <v>2.44</v>
       </c>
-      <c r="I20" s="30" t="s">
+      <c r="I20" s="27" t="s">
         <v>219</v>
       </c>
-      <c r="J20" s="31">
+      <c r="J20" s="37">
         <v>8.2075000000000014</v>
       </c>
-      <c r="K20" s="32">
+      <c r="K20" s="38">
         <v>16.226249999999997</v>
       </c>
-      <c r="L20" s="33">
+      <c r="L20" s="39">
         <v>11.477862766125</v>
       </c>
     </row>
@@ -10749,16 +10759,16 @@
       <c r="G21" s="18">
         <v>5.7</v>
       </c>
-      <c r="I21" s="30" t="s">
+      <c r="I21" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="J21" s="31">
+      <c r="J21" s="37">
         <v>6.0833333333333321</v>
       </c>
-      <c r="K21" s="32">
+      <c r="K21" s="38">
         <v>15.586666666666668</v>
       </c>
-      <c r="L21" s="33">
+      <c r="L21" s="39">
         <v>10.361629527000002</v>
       </c>
     </row>
@@ -10784,16 +10794,16 @@
       <c r="G22" s="18">
         <v>16.21</v>
       </c>
-      <c r="I22" s="30" t="s">
+      <c r="I22" s="27" t="s">
         <v>221</v>
       </c>
-      <c r="J22" s="31">
+      <c r="J22" s="37">
         <v>6.7061999999999999</v>
       </c>
-      <c r="K22" s="32">
+      <c r="K22" s="38">
         <v>16.212800000000001</v>
       </c>
-      <c r="L22" s="33">
+      <c r="L22" s="39">
         <v>10.959806601866665</v>
       </c>
     </row>
@@ -10819,16 +10829,16 @@
       <c r="G23" s="18">
         <v>13.51</v>
       </c>
-      <c r="I23" s="30" t="s">
+      <c r="I23" s="27" t="s">
         <v>222</v>
       </c>
-      <c r="J23" s="31">
+      <c r="J23" s="37">
         <v>6.6417999999999999</v>
       </c>
-      <c r="K23" s="32">
+      <c r="K23" s="38">
         <v>16.791266666666665</v>
       </c>
-      <c r="L23" s="33">
+      <c r="L23" s="39">
         <v>10.897679031399999</v>
       </c>
     </row>
@@ -10854,16 +10864,16 @@
       <c r="G24" s="18">
         <v>16.3</v>
       </c>
-      <c r="I24" s="30" t="s">
+      <c r="I24" s="27" t="s">
         <v>223</v>
       </c>
-      <c r="J24" s="31">
+      <c r="J24" s="37">
         <v>7.9019999999999984</v>
       </c>
-      <c r="K24" s="32">
+      <c r="K24" s="38">
         <v>15.073333333333331</v>
       </c>
-      <c r="L24" s="33">
+      <c r="L24" s="39">
         <v>11.354973077066665</v>
       </c>
     </row>
@@ -10889,16 +10899,16 @@
       <c r="G25" s="18">
         <v>15.31</v>
       </c>
-      <c r="I25" s="30" t="s">
+      <c r="I25" s="27" t="s">
         <v>224</v>
       </c>
-      <c r="J25" s="31">
+      <c r="J25" s="37">
         <v>6.9156295574666675</v>
       </c>
-      <c r="K25" s="32">
+      <c r="K25" s="38">
         <v>16.508156901400003</v>
       </c>
-      <c r="L25" s="33">
+      <c r="L25" s="39">
         <v>11.035834536666666</v>
       </c>
     </row>
@@ -10924,16 +10934,16 @@
       <c r="G26" s="18">
         <v>15.06</v>
       </c>
-      <c r="I26" s="30" t="s">
+      <c r="I26" s="27" t="s">
         <v>225</v>
       </c>
-      <c r="J26" s="31">
+      <c r="J26" s="37">
         <v>5.8515384615384622</v>
       </c>
-      <c r="K26" s="32">
+      <c r="K26" s="38">
         <v>14.074615384615383</v>
       </c>
-      <c r="L26" s="33">
+      <c r="L26" s="39">
         <v>9.2440913864615375</v>
       </c>
     </row>
@@ -10959,12 +10969,12 @@
       <c r="G27" s="18">
         <v>14.11</v>
       </c>
-      <c r="I27" s="30" t="s">
+      <c r="I27" s="27" t="s">
         <v>305</v>
       </c>
-      <c r="J27" s="31"/>
-      <c r="K27" s="32"/>
-      <c r="L27" s="33"/>
+      <c r="J27" s="37"/>
+      <c r="K27" s="38"/>
+      <c r="L27" s="39"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="17" t="s">
@@ -10988,16 +10998,16 @@
       <c r="G28" s="18">
         <v>13.34</v>
       </c>
-      <c r="I28" s="34" t="s">
+      <c r="I28" s="28" t="s">
         <v>226</v>
       </c>
-      <c r="J28" s="35">
+      <c r="J28" s="40">
         <v>6.8046156568829819</v>
       </c>
-      <c r="K28" s="36">
+      <c r="K28" s="41">
         <v>16.033338791049651</v>
       </c>
-      <c r="L28" s="37">
+      <c r="L28" s="42">
         <v>10.746023539205673</v>
       </c>
     </row>

</xml_diff>